<commit_message>
AML (マウスレイヤー) を Ctrl / Shift / Win / Alt で解除する (#22)
これまでは修飾キーの位置 (A / - / Z / / / Win / Alt) を AML の excluded-positions に
入れ、MOUSE_MOVE ではそこを Ctrl / Shift / Win / Alt にしていた。そのため、マウスを
使った直後 (AML 中) に A / Z / - / / をタップすると、文字が入らず修飾キーのタップに
なっていた。

- excluded-positions を D / K (&mo SCRL) だけにする。修飾キーの位置を押すと AML が切れる
- MOUSE_MOVE の修飾キーの位置を &trans にする (BASE と同じ &mt / &kp。タップで文字、
  長押しで修飾キー)。ZMK v0.3.0 では zip_temp_layer のリスナーが keymap より先に
  レイヤーを切るので、どちらにしても BASE のキーになるが、&trans で意図を明示する
- MOUSE_SCROLL の修飾キーはそのまま。修飾キーとクリック・ホイールを組み合わせるときは
  D / K を押してから修飾キーを押す (例: D → Z → F で Shift + クリック)
- KEYMAP.html / KEYMAP.xlsx を作り直す

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QFG6t92cGtjhGTDoN62Yvg
</commit_message>
<xml_diff>
--- a/KEYMAP.xlsx
+++ b/KEYMAP.xlsx
@@ -5332,7 +5332,7 @@
       <c r="B97" s="7" t="inlineStr">
         <is>
           <t>pos 10
-&amp;kp LCTRL</t>
+&amp;trans</t>
         </is>
       </c>
       <c r="C97" s="7" t="inlineStr">
@@ -5389,7 +5389,7 @@
       <c r="N97" s="7" t="inlineStr">
         <is>
           <t>pos 19
-&amp;kp RCTRL</t>
+&amp;trans</t>
         </is>
       </c>
     </row>
@@ -5401,7 +5401,7 @@
       </c>
       <c r="B98" s="9" t="inlineStr">
         <is>
-          <t>LCtrl</t>
+          <t>▽</t>
         </is>
       </c>
       <c r="C98" s="9" t="inlineStr"/>
@@ -5425,7 +5425,7 @@
       <c r="M98" s="9" t="inlineStr"/>
       <c r="N98" s="9" t="inlineStr">
         <is>
-          <t>RCtrl</t>
+          <t>▽</t>
         </is>
       </c>
     </row>
@@ -5438,7 +5438,7 @@
       <c r="B99" s="7" t="inlineStr">
         <is>
           <t>pos 20
-&amp;kp LEFT_SHIFT</t>
+&amp;trans</t>
         </is>
       </c>
       <c r="C99" s="7" t="inlineStr">
@@ -5495,7 +5495,7 @@
       <c r="N99" s="7" t="inlineStr">
         <is>
           <t>pos 29
-&amp;kp RIGHT_SHIFT</t>
+&amp;trans</t>
         </is>
       </c>
     </row>
@@ -5507,7 +5507,7 @@
       </c>
       <c r="B100" s="9" t="inlineStr">
         <is>
-          <t>LShift</t>
+          <t>▽</t>
         </is>
       </c>
       <c r="C100" s="9" t="inlineStr"/>
@@ -5523,7 +5523,7 @@
       <c r="M100" s="9" t="inlineStr"/>
       <c r="N100" s="9" t="inlineStr">
         <is>
-          <t>RShift</t>
+          <t>▽</t>
         </is>
       </c>
     </row>
@@ -5542,13 +5542,13 @@
       <c r="C101" s="7" t="inlineStr">
         <is>
           <t>pos 31
-&amp;kp LEFT_WIN</t>
+&amp;trans</t>
         </is>
       </c>
       <c r="D101" s="7" t="inlineStr">
         <is>
           <t>pos 32
-&amp;kp LEFT_ALT</t>
+&amp;trans</t>
         </is>
       </c>
       <c r="E101" s="7" t="inlineStr">
@@ -5616,12 +5616,12 @@
       <c r="B102" s="9" t="inlineStr"/>
       <c r="C102" s="9" t="inlineStr">
         <is>
-          <t>LWin</t>
+          <t>▽</t>
         </is>
       </c>
       <c r="D102" s="9" t="inlineStr">
         <is>
-          <t>LAlt</t>
+          <t>▽</t>
         </is>
       </c>
       <c r="E102" s="9" t="inlineStr"/>
@@ -10950,7 +10950,7 @@
       <c r="B97" s="7" t="inlineStr">
         <is>
           <t>pos 10
-&amp;kp LCTRL</t>
+&amp;trans</t>
         </is>
       </c>
       <c r="C97" s="7" t="inlineStr">
@@ -11007,7 +11007,7 @@
       <c r="N97" s="7" t="inlineStr">
         <is>
           <t>pos 19
-&amp;kp RCTRL</t>
+&amp;trans</t>
         </is>
       </c>
     </row>
@@ -11019,7 +11019,7 @@
       </c>
       <c r="B98" s="9" t="inlineStr">
         <is>
-          <t>&amp;kp LCTRL</t>
+          <t>▽</t>
         </is>
       </c>
       <c r="C98" s="9" t="inlineStr"/>
@@ -11043,7 +11043,7 @@
       <c r="M98" s="9" t="inlineStr"/>
       <c r="N98" s="9" t="inlineStr">
         <is>
-          <t>&amp;kp RCTRL</t>
+          <t>▽</t>
         </is>
       </c>
     </row>
@@ -11056,7 +11056,7 @@
       <c r="B99" s="7" t="inlineStr">
         <is>
           <t>pos 20
-&amp;kp LEFT_SHIFT</t>
+&amp;trans</t>
         </is>
       </c>
       <c r="C99" s="7" t="inlineStr">
@@ -11113,7 +11113,7 @@
       <c r="N99" s="7" t="inlineStr">
         <is>
           <t>pos 29
-&amp;kp RIGHT_SHIFT</t>
+&amp;trans</t>
         </is>
       </c>
     </row>
@@ -11125,7 +11125,7 @@
       </c>
       <c r="B100" s="9" t="inlineStr">
         <is>
-          <t>&amp;kp LEFT_SHIFT</t>
+          <t>▽</t>
         </is>
       </c>
       <c r="C100" s="9" t="inlineStr"/>
@@ -11141,7 +11141,7 @@
       <c r="M100" s="9" t="inlineStr"/>
       <c r="N100" s="9" t="inlineStr">
         <is>
-          <t>&amp;kp RIGHT_SHIFT</t>
+          <t>▽</t>
         </is>
       </c>
     </row>
@@ -11160,13 +11160,13 @@
       <c r="C101" s="7" t="inlineStr">
         <is>
           <t>pos 31
-&amp;kp LEFT_WIN</t>
+&amp;trans</t>
         </is>
       </c>
       <c r="D101" s="7" t="inlineStr">
         <is>
           <t>pos 32
-&amp;kp LEFT_ALT</t>
+&amp;trans</t>
         </is>
       </c>
       <c r="E101" s="7" t="inlineStr">
@@ -11234,12 +11234,12 @@
       <c r="B102" s="9" t="inlineStr"/>
       <c r="C102" s="9" t="inlineStr">
         <is>
-          <t>&amp;kp LEFT_WIN</t>
+          <t>▽</t>
         </is>
       </c>
       <c r="D102" s="9" t="inlineStr">
         <is>
-          <t>&amp;kp LEFT_ALT</t>
+          <t>▽</t>
         </is>
       </c>
       <c r="E102" s="9" t="inlineStr"/>

</xml_diff>